<commit_message>
feat: mobile PWA (responsive UI + manifest + service worker)
</commit_message>
<xml_diff>
--- a/db/DB_수사종결까지.xlsx
+++ b/db/DB_수사종결까지.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\songjoo\Documents\GitHub\word-game\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D66877F8-1C33-48FB-8085-F28568F65329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AB4BBA-1230-48B2-91C9-FFE9C86E024E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{5A5E7394-FEFB-4E15-8D3D-4FA3946DC3B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{5A5E7394-FEFB-4E15-8D3D-4FA3946DC3B9}"/>
   </bookViews>
   <sheets>
     <sheet name="관할 및 제척기피" sheetId="1" r:id="rId1"/>

</xml_diff>